<commit_message>
test(parse): give the BMO duplicate-lines fixture valid ISINs
</commit_message>
<xml_diff>
--- a/tests/fixtures/issuers/bmo/duplicate_lines.xlsx
+++ b/tests/fixtures/issuers/bmo/duplicate_lines.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Holdings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CA000000BB11</t>
+          <t>CA000000BB16</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -541,7 +541,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RU0000000001</t>
+          <t>RU0000000003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>RU0000000001</t>
+          <t>RU0000000003</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">

</xml_diff>